<commit_message>
translated study 1 condition assignment to german
</commit_message>
<xml_diff>
--- a/method/study 1/organiser/Study 1 Condition Assignment Sheet.xlsx
+++ b/method/study 1/organiser/Study 1 Condition Assignment Sheet.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Ian/git/ironic-effect-of-thought-suppression-replication/blind materials fixed/Study 1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Ian/git/ironic-effect-of-thought-suppression-replication/method/study 1/organiser/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4A107D8-A108-4D4D-BFFB-2F63E893221B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BFDA3AD-E18E-7B46-A6AB-D4C5DA067147}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="33660" windowHeight="19600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -72,30 +72,6 @@
   </si>
   <si>
     <t>Tick when completed, following the instructions in "Study 1 Researcher instructions.docx"</t>
-  </si>
-  <si>
-    <t>For your first task, please try to think about a MOUNTAIN for the next five minutes. I will be back in five minutes</t>
-  </si>
-  <si>
-    <t>For your first task, please try to think about a CHILD for the next five minutes. I will be back in five minutes</t>
-  </si>
-  <si>
-    <t>For your first task, please try NOT to think about a CHILD for the next five minutes. I will be back in five minutes</t>
-  </si>
-  <si>
-    <t>For your first task, please try to think about a HOUSE for the next five minutes. I will be back in five minutes</t>
-  </si>
-  <si>
-    <t>For your first task, please try NOT to think about a CAR for the next five minutes. I will be back in five minutes</t>
-  </si>
-  <si>
-    <t>For your first task, please try NOT to think about a HOUSE for the next five minutes. I will be back in five minutes</t>
-  </si>
-  <si>
-    <t>For your first task, please try NOT to think about a MOUNTAIN for the next five minutes. I will be back in five minutes</t>
-  </si>
-  <si>
-    <t>For your first task, please try to think about a CAR for the next five minutes. I will be back in five minutes</t>
   </si>
   <si>
     <t>Notes</t>
@@ -167,12 +143,36 @@
   <si>
     <t>random 1-2. 1 = "try NOT", 2 = "try".</t>
   </si>
+  <si>
+    <t>Versuchen Sie bei Ihrer ersten Aufgabe, in den nächsten fünf Minuten an einen BERG zu denken. Ich bin in fünf Minuten zurück.</t>
+  </si>
+  <si>
+    <t>Versuchen Sie bei Ihrer ersten Aufgabe, in den nächsten fünf Minuten an ein KIND zu denken. Ich bin in fünf Minuten zurück.</t>
+  </si>
+  <si>
+    <t>Versuchen Sie bei Ihrer ersten Aufgabe, in den nächsten fünf Minuten NICHT an ein KIND zu denken. Ich bin in fünf Minuten zurück.</t>
+  </si>
+  <si>
+    <t>Versuchen Sie bei Ihrer ersten Aufgabe, in den nächsten fünf Minuten an ein HAUS zu denken. Ich bin in fünf Minuten zurück.</t>
+  </si>
+  <si>
+    <t>Versuchen Sie bei Ihrer ersten Aufgabe, in den nächsten fünf Minuten NICHT an ein AUTO zu denken. Ich bin in fünf Minuten zurück.</t>
+  </si>
+  <si>
+    <t>Versuchen Sie bei Ihrer ersten Aufgabe, in den nächsten fünf Minuten NICHT an ein HAUS zu denken. Ich bin in fünf Minuten zurück.</t>
+  </si>
+  <si>
+    <t>Versuchen Sie bei Ihrer ersten Aufgabe, in den nächsten fünf Minuten NICHT an einen BERG zu denken. Ich bin in fünf Minuten zurück.</t>
+  </si>
+  <si>
+    <t>Versuchen Sie bei Ihrer ersten Aufgabe, in den nächsten fünf Minuten an ein AUTO zu denken. Ich bin in fünf Minuten zurück.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -196,6 +196,12 @@
     <font>
       <sz val="11"/>
       <name val="Calibri (Body)"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -239,7 +245,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -261,6 +267,7 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -545,7 +552,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.83203125" style="1"/>
-    <col min="2" max="2" width="89.33203125" style="4" customWidth="1"/>
+    <col min="2" max="2" width="107.6640625" style="4" customWidth="1"/>
     <col min="3" max="3" width="12.5" customWidth="1"/>
     <col min="4" max="4" width="12.1640625" customWidth="1"/>
     <col min="5" max="5" width="22.5" style="4" customWidth="1"/>
@@ -578,22 +585,22 @@
     </row>
     <row r="2" spans="1:7" s="2" customFormat="1" ht="96" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="G2" s="3" t="s">
         <v>8</v>
@@ -603,8 +610,8 @@
       <c r="A3" s="5">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
-        <v>9</v>
+      <c r="B3" s="9" t="s">
+        <v>14</v>
       </c>
       <c r="C3">
         <v>2</v>
@@ -624,8 +631,8 @@
       <c r="A4" s="5">
         <v>2</v>
       </c>
-      <c r="B4" t="s">
-        <v>10</v>
+      <c r="B4" s="9" t="s">
+        <v>15</v>
       </c>
       <c r="C4">
         <v>2</v>
@@ -645,8 +652,8 @@
       <c r="A5" s="5">
         <v>3</v>
       </c>
-      <c r="B5" t="s">
-        <v>11</v>
+      <c r="B5" s="9" t="s">
+        <v>16</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -666,8 +673,8 @@
       <c r="A6" s="5">
         <v>4</v>
       </c>
-      <c r="B6" t="s">
-        <v>12</v>
+      <c r="B6" s="9" t="s">
+        <v>17</v>
       </c>
       <c r="C6">
         <v>2</v>
@@ -687,8 +694,8 @@
       <c r="A7" s="5">
         <v>5</v>
       </c>
-      <c r="B7" t="s">
-        <v>13</v>
+      <c r="B7" s="9" t="s">
+        <v>18</v>
       </c>
       <c r="C7">
         <v>1</v>
@@ -708,8 +715,8 @@
       <c r="A8" s="5">
         <v>6</v>
       </c>
-      <c r="B8" t="s">
-        <v>12</v>
+      <c r="B8" s="9" t="s">
+        <v>17</v>
       </c>
       <c r="C8">
         <v>2</v>
@@ -729,8 +736,8 @@
       <c r="A9" s="5">
         <v>7</v>
       </c>
-      <c r="B9" t="s">
-        <v>9</v>
+      <c r="B9" s="9" t="s">
+        <v>14</v>
       </c>
       <c r="C9">
         <v>2</v>
@@ -750,8 +757,8 @@
       <c r="A10" s="5">
         <v>8</v>
       </c>
-      <c r="B10" t="s">
-        <v>11</v>
+      <c r="B10" s="9" t="s">
+        <v>16</v>
       </c>
       <c r="C10">
         <v>1</v>
@@ -771,8 +778,8 @@
       <c r="A11" s="5">
         <v>9</v>
       </c>
-      <c r="B11" t="s">
-        <v>12</v>
+      <c r="B11" s="9" t="s">
+        <v>17</v>
       </c>
       <c r="C11">
         <v>2</v>
@@ -792,8 +799,8 @@
       <c r="A12" s="5">
         <v>10</v>
       </c>
-      <c r="B12" t="s">
-        <v>14</v>
+      <c r="B12" s="9" t="s">
+        <v>19</v>
       </c>
       <c r="C12">
         <v>1</v>
@@ -813,8 +820,8 @@
       <c r="A13" s="5">
         <v>11</v>
       </c>
-      <c r="B13" t="s">
-        <v>13</v>
+      <c r="B13" s="9" t="s">
+        <v>18</v>
       </c>
       <c r="C13">
         <v>1</v>
@@ -834,8 +841,8 @@
       <c r="A14" s="5">
         <v>12</v>
       </c>
-      <c r="B14" t="s">
-        <v>11</v>
+      <c r="B14" s="9" t="s">
+        <v>16</v>
       </c>
       <c r="C14">
         <v>1</v>
@@ -855,8 +862,8 @@
       <c r="A15" s="5">
         <v>13</v>
       </c>
-      <c r="B15" t="s">
-        <v>15</v>
+      <c r="B15" s="9" t="s">
+        <v>20</v>
       </c>
       <c r="C15">
         <v>1</v>
@@ -876,8 +883,8 @@
       <c r="A16" s="5">
         <v>14</v>
       </c>
-      <c r="B16" t="s">
-        <v>9</v>
+      <c r="B16" s="9" t="s">
+        <v>14</v>
       </c>
       <c r="C16">
         <v>2</v>
@@ -897,8 +904,8 @@
       <c r="A17" s="5">
         <v>15</v>
       </c>
-      <c r="B17" t="s">
-        <v>11</v>
+      <c r="B17" s="9" t="s">
+        <v>16</v>
       </c>
       <c r="C17">
         <v>1</v>
@@ -918,8 +925,8 @@
       <c r="A18" s="5">
         <v>16</v>
       </c>
-      <c r="B18" t="s">
-        <v>14</v>
+      <c r="B18" s="9" t="s">
+        <v>19</v>
       </c>
       <c r="C18">
         <v>1</v>
@@ -939,8 +946,8 @@
       <c r="A19" s="5">
         <v>17</v>
       </c>
-      <c r="B19" t="s">
-        <v>12</v>
+      <c r="B19" s="9" t="s">
+        <v>17</v>
       </c>
       <c r="C19">
         <v>2</v>
@@ -960,8 +967,8 @@
       <c r="A20" s="5">
         <v>18</v>
       </c>
-      <c r="B20" t="s">
-        <v>14</v>
+      <c r="B20" s="9" t="s">
+        <v>19</v>
       </c>
       <c r="C20">
         <v>1</v>
@@ -981,8 +988,8 @@
       <c r="A21" s="5">
         <v>19</v>
       </c>
-      <c r="B21" t="s">
-        <v>9</v>
+      <c r="B21" s="9" t="s">
+        <v>14</v>
       </c>
       <c r="C21">
         <v>2</v>
@@ -1002,8 +1009,8 @@
       <c r="A22" s="1">
         <v>20</v>
       </c>
-      <c r="B22" t="s">
-        <v>15</v>
+      <c r="B22" s="9" t="s">
+        <v>20</v>
       </c>
       <c r="C22">
         <v>1</v>
@@ -1023,8 +1030,8 @@
       <c r="A23" s="1">
         <v>21</v>
       </c>
-      <c r="B23" t="s">
-        <v>10</v>
+      <c r="B23" s="9" t="s">
+        <v>15</v>
       </c>
       <c r="C23">
         <v>2</v>
@@ -1044,8 +1051,8 @@
       <c r="A24" s="1">
         <v>22</v>
       </c>
-      <c r="B24" t="s">
-        <v>14</v>
+      <c r="B24" s="9" t="s">
+        <v>19</v>
       </c>
       <c r="C24">
         <v>1</v>
@@ -1065,8 +1072,8 @@
       <c r="A25" s="1">
         <v>23</v>
       </c>
-      <c r="B25" t="s">
-        <v>11</v>
+      <c r="B25" s="9" t="s">
+        <v>16</v>
       </c>
       <c r="C25">
         <v>1</v>
@@ -1086,8 +1093,8 @@
       <c r="A26" s="1">
         <v>24</v>
       </c>
-      <c r="B26" t="s">
-        <v>14</v>
+      <c r="B26" s="9" t="s">
+        <v>19</v>
       </c>
       <c r="C26">
         <v>1</v>
@@ -1107,8 +1114,8 @@
       <c r="A27" s="1">
         <v>25</v>
       </c>
-      <c r="B27" t="s">
-        <v>10</v>
+      <c r="B27" s="9" t="s">
+        <v>15</v>
       </c>
       <c r="C27">
         <v>2</v>
@@ -1128,8 +1135,8 @@
       <c r="A28" s="1">
         <v>26</v>
       </c>
-      <c r="B28" t="s">
-        <v>14</v>
+      <c r="B28" s="9" t="s">
+        <v>19</v>
       </c>
       <c r="C28">
         <v>1</v>
@@ -1149,8 +1156,8 @@
       <c r="A29" s="1">
         <v>27</v>
       </c>
-      <c r="B29" t="s">
-        <v>9</v>
+      <c r="B29" s="9" t="s">
+        <v>14</v>
       </c>
       <c r="C29">
         <v>2</v>
@@ -1170,8 +1177,8 @@
       <c r="A30" s="1">
         <v>28</v>
       </c>
-      <c r="B30" t="s">
-        <v>12</v>
+      <c r="B30" s="9" t="s">
+        <v>17</v>
       </c>
       <c r="C30">
         <v>2</v>
@@ -1191,8 +1198,8 @@
       <c r="A31" s="1">
         <v>29</v>
       </c>
-      <c r="B31" t="s">
-        <v>11</v>
+      <c r="B31" s="9" t="s">
+        <v>16</v>
       </c>
       <c r="C31">
         <v>1</v>
@@ -1212,8 +1219,8 @@
       <c r="A32" s="1">
         <v>30</v>
       </c>
-      <c r="B32" t="s">
-        <v>9</v>
+      <c r="B32" s="9" t="s">
+        <v>14</v>
       </c>
       <c r="C32">
         <v>2</v>
@@ -1233,8 +1240,8 @@
       <c r="A33" s="1">
         <v>31</v>
       </c>
-      <c r="B33" t="s">
-        <v>13</v>
+      <c r="B33" s="9" t="s">
+        <v>18</v>
       </c>
       <c r="C33">
         <v>1</v>
@@ -1254,8 +1261,8 @@
       <c r="A34" s="1">
         <v>32</v>
       </c>
-      <c r="B34" t="s">
-        <v>11</v>
+      <c r="B34" s="9" t="s">
+        <v>16</v>
       </c>
       <c r="C34">
         <v>1</v>
@@ -1275,8 +1282,8 @@
       <c r="A35" s="1">
         <v>33</v>
       </c>
-      <c r="B35" t="s">
-        <v>15</v>
+      <c r="B35" s="9" t="s">
+        <v>20</v>
       </c>
       <c r="C35">
         <v>1</v>
@@ -1296,8 +1303,8 @@
       <c r="A36" s="1">
         <v>34</v>
       </c>
-      <c r="B36" t="s">
-        <v>12</v>
+      <c r="B36" s="9" t="s">
+        <v>17</v>
       </c>
       <c r="C36">
         <v>2</v>
@@ -1317,8 +1324,8 @@
       <c r="A37" s="1">
         <v>35</v>
       </c>
-      <c r="B37" t="s">
-        <v>15</v>
+      <c r="B37" s="9" t="s">
+        <v>20</v>
       </c>
       <c r="C37">
         <v>1</v>
@@ -1338,8 +1345,8 @@
       <c r="A38" s="1">
         <v>36</v>
       </c>
-      <c r="B38" t="s">
-        <v>12</v>
+      <c r="B38" s="9" t="s">
+        <v>17</v>
       </c>
       <c r="C38">
         <v>2</v>
@@ -1359,8 +1366,8 @@
       <c r="A39" s="1">
         <v>37</v>
       </c>
-      <c r="B39" t="s">
-        <v>12</v>
+      <c r="B39" s="9" t="s">
+        <v>17</v>
       </c>
       <c r="C39">
         <v>2</v>
@@ -1380,8 +1387,8 @@
       <c r="A40" s="1">
         <v>38</v>
       </c>
-      <c r="B40" t="s">
-        <v>16</v>
+      <c r="B40" s="9" t="s">
+        <v>21</v>
       </c>
       <c r="C40">
         <v>2</v>
@@ -1401,8 +1408,8 @@
       <c r="A41" s="1">
         <v>39</v>
       </c>
-      <c r="B41" t="s">
-        <v>10</v>
+      <c r="B41" s="9" t="s">
+        <v>15</v>
       </c>
       <c r="C41">
         <v>2</v>
@@ -1422,8 +1429,8 @@
       <c r="A42" s="1">
         <v>40</v>
       </c>
-      <c r="B42" t="s">
-        <v>9</v>
+      <c r="B42" s="9" t="s">
+        <v>14</v>
       </c>
       <c r="C42">
         <v>2</v>
@@ -1443,8 +1450,8 @@
       <c r="A43" s="1">
         <v>41</v>
       </c>
-      <c r="B43" t="s">
-        <v>16</v>
+      <c r="B43" s="9" t="s">
+        <v>21</v>
       </c>
       <c r="C43">
         <v>2</v>
@@ -1464,8 +1471,8 @@
       <c r="A44" s="1">
         <v>42</v>
       </c>
-      <c r="B44" t="s">
-        <v>14</v>
+      <c r="B44" s="9" t="s">
+        <v>19</v>
       </c>
       <c r="C44">
         <v>1</v>
@@ -1485,8 +1492,8 @@
       <c r="A45" s="1">
         <v>43</v>
       </c>
-      <c r="B45" t="s">
-        <v>16</v>
+      <c r="B45" s="9" t="s">
+        <v>21</v>
       </c>
       <c r="C45">
         <v>2</v>
@@ -1506,8 +1513,8 @@
       <c r="A46" s="1">
         <v>44</v>
       </c>
-      <c r="B46" t="s">
-        <v>11</v>
+      <c r="B46" s="9" t="s">
+        <v>16</v>
       </c>
       <c r="C46">
         <v>1</v>
@@ -1527,8 +1534,8 @@
       <c r="A47" s="1">
         <v>45</v>
       </c>
-      <c r="B47" t="s">
-        <v>10</v>
+      <c r="B47" s="9" t="s">
+        <v>15</v>
       </c>
       <c r="C47">
         <v>2</v>
@@ -1548,8 +1555,8 @@
       <c r="A48" s="1">
         <v>46</v>
       </c>
-      <c r="B48" t="s">
-        <v>15</v>
+      <c r="B48" s="9" t="s">
+        <v>20</v>
       </c>
       <c r="C48">
         <v>1</v>
@@ -1569,8 +1576,8 @@
       <c r="A49" s="1">
         <v>47</v>
       </c>
-      <c r="B49" t="s">
-        <v>14</v>
+      <c r="B49" s="9" t="s">
+        <v>19</v>
       </c>
       <c r="C49">
         <v>1</v>
@@ -1590,8 +1597,8 @@
       <c r="A50" s="1">
         <v>48</v>
       </c>
-      <c r="B50" t="s">
-        <v>15</v>
+      <c r="B50" s="9" t="s">
+        <v>20</v>
       </c>
       <c r="C50">
         <v>1</v>
@@ -1611,8 +1618,8 @@
       <c r="A51" s="1">
         <v>49</v>
       </c>
-      <c r="B51" t="s">
-        <v>16</v>
+      <c r="B51" s="9" t="s">
+        <v>21</v>
       </c>
       <c r="C51">
         <v>2</v>
@@ -1632,8 +1639,8 @@
       <c r="A52" s="1">
         <v>50</v>
       </c>
-      <c r="B52" t="s">
-        <v>16</v>
+      <c r="B52" s="9" t="s">
+        <v>21</v>
       </c>
       <c r="C52">
         <v>2</v>
@@ -1653,8 +1660,8 @@
       <c r="A53" s="1">
         <v>51</v>
       </c>
-      <c r="B53" t="s">
-        <v>10</v>
+      <c r="B53" s="9" t="s">
+        <v>15</v>
       </c>
       <c r="C53">
         <v>2</v>
@@ -1674,8 +1681,8 @@
       <c r="A54" s="1">
         <v>52</v>
       </c>
-      <c r="B54" t="s">
-        <v>11</v>
+      <c r="B54" s="9" t="s">
+        <v>16</v>
       </c>
       <c r="C54">
         <v>1</v>
@@ -1695,8 +1702,8 @@
       <c r="A55" s="1">
         <v>53</v>
       </c>
-      <c r="B55" t="s">
-        <v>16</v>
+      <c r="B55" s="9" t="s">
+        <v>21</v>
       </c>
       <c r="C55">
         <v>2</v>
@@ -1716,8 +1723,8 @@
       <c r="A56" s="1">
         <v>54</v>
       </c>
-      <c r="B56" t="s">
-        <v>10</v>
+      <c r="B56" s="9" t="s">
+        <v>15</v>
       </c>
       <c r="C56">
         <v>2</v>
@@ -1737,8 +1744,8 @@
       <c r="A57" s="1">
         <v>55</v>
       </c>
-      <c r="B57" t="s">
-        <v>16</v>
+      <c r="B57" s="9" t="s">
+        <v>21</v>
       </c>
       <c r="C57">
         <v>2</v>
@@ -1758,8 +1765,8 @@
       <c r="A58" s="1">
         <v>56</v>
       </c>
-      <c r="B58" t="s">
-        <v>15</v>
+      <c r="B58" s="9" t="s">
+        <v>20</v>
       </c>
       <c r="C58">
         <v>1</v>
@@ -1779,8 +1786,8 @@
       <c r="A59" s="1">
         <v>57</v>
       </c>
-      <c r="B59" t="s">
-        <v>9</v>
+      <c r="B59" s="9" t="s">
+        <v>14</v>
       </c>
       <c r="C59">
         <v>2</v>
@@ -1800,8 +1807,8 @@
       <c r="A60" s="1">
         <v>58</v>
       </c>
-      <c r="B60" t="s">
-        <v>16</v>
+      <c r="B60" s="9" t="s">
+        <v>21</v>
       </c>
       <c r="C60">
         <v>2</v>
@@ -1821,8 +1828,8 @@
       <c r="A61" s="1">
         <v>59</v>
       </c>
-      <c r="B61" t="s">
-        <v>15</v>
+      <c r="B61" s="9" t="s">
+        <v>20</v>
       </c>
       <c r="C61">
         <v>1</v>
@@ -1842,8 +1849,8 @@
       <c r="A62" s="1">
         <v>60</v>
       </c>
-      <c r="B62" t="s">
-        <v>13</v>
+      <c r="B62" s="9" t="s">
+        <v>18</v>
       </c>
       <c r="C62">
         <v>1</v>
@@ -1863,8 +1870,8 @@
       <c r="A63" s="1">
         <v>61</v>
       </c>
-      <c r="B63" t="s">
-        <v>15</v>
+      <c r="B63" s="9" t="s">
+        <v>20</v>
       </c>
       <c r="C63">
         <v>1</v>
@@ -1884,8 +1891,8 @@
       <c r="A64" s="1">
         <v>62</v>
       </c>
-      <c r="B64" t="s">
-        <v>10</v>
+      <c r="B64" s="9" t="s">
+        <v>15</v>
       </c>
       <c r="C64">
         <v>2</v>
@@ -1905,8 +1912,8 @@
       <c r="A65" s="1">
         <v>63</v>
       </c>
-      <c r="B65" t="s">
-        <v>13</v>
+      <c r="B65" s="9" t="s">
+        <v>18</v>
       </c>
       <c r="C65">
         <v>1</v>
@@ -1926,8 +1933,8 @@
       <c r="A66" s="1">
         <v>64</v>
       </c>
-      <c r="B66" t="s">
-        <v>12</v>
+      <c r="B66" s="9" t="s">
+        <v>17</v>
       </c>
       <c r="C66">
         <v>2</v>
@@ -1947,8 +1954,8 @@
       <c r="A67" s="1">
         <v>65</v>
       </c>
-      <c r="B67" t="s">
-        <v>15</v>
+      <c r="B67" s="9" t="s">
+        <v>20</v>
       </c>
       <c r="C67">
         <v>1</v>
@@ -1968,8 +1975,8 @@
       <c r="A68" s="1">
         <v>66</v>
       </c>
-      <c r="B68" t="s">
-        <v>9</v>
+      <c r="B68" s="9" t="s">
+        <v>14</v>
       </c>
       <c r="C68">
         <v>2</v>
@@ -1989,8 +1996,8 @@
       <c r="A69" s="1">
         <v>67</v>
       </c>
-      <c r="B69" t="s">
-        <v>13</v>
+      <c r="B69" s="9" t="s">
+        <v>18</v>
       </c>
       <c r="C69">
         <v>1</v>
@@ -2010,8 +2017,8 @@
       <c r="A70" s="1">
         <v>68</v>
       </c>
-      <c r="B70" t="s">
-        <v>13</v>
+      <c r="B70" s="9" t="s">
+        <v>18</v>
       </c>
       <c r="C70">
         <v>1</v>
@@ -2031,8 +2038,8 @@
       <c r="A71" s="1">
         <v>69</v>
       </c>
-      <c r="B71" t="s">
-        <v>13</v>
+      <c r="B71" s="9" t="s">
+        <v>18</v>
       </c>
       <c r="C71">
         <v>1</v>
@@ -2052,8 +2059,8 @@
       <c r="A72" s="1">
         <v>70</v>
       </c>
-      <c r="B72" t="s">
-        <v>13</v>
+      <c r="B72" s="9" t="s">
+        <v>18</v>
       </c>
       <c r="C72">
         <v>1</v>
@@ -2073,8 +2080,8 @@
       <c r="A73" s="1">
         <v>71</v>
       </c>
-      <c r="B73" t="s">
-        <v>10</v>
+      <c r="B73" s="9" t="s">
+        <v>15</v>
       </c>
       <c r="C73">
         <v>2</v>
@@ -2094,8 +2101,8 @@
       <c r="A74" s="1">
         <v>72</v>
       </c>
-      <c r="B74" t="s">
-        <v>10</v>
+      <c r="B74" s="9" t="s">
+        <v>15</v>
       </c>
       <c r="C74">
         <v>2</v>
@@ -2115,8 +2122,8 @@
       <c r="A75" s="1">
         <v>73</v>
       </c>
-      <c r="B75" t="s">
-        <v>9</v>
+      <c r="B75" s="9" t="s">
+        <v>14</v>
       </c>
       <c r="C75">
         <v>2</v>
@@ -2136,8 +2143,8 @@
       <c r="A76" s="1">
         <v>74</v>
       </c>
-      <c r="B76" t="s">
-        <v>12</v>
+      <c r="B76" s="9" t="s">
+        <v>17</v>
       </c>
       <c r="C76">
         <v>2</v>
@@ -2157,8 +2164,8 @@
       <c r="A77" s="1">
         <v>75</v>
       </c>
-      <c r="B77" t="s">
-        <v>13</v>
+      <c r="B77" s="9" t="s">
+        <v>18</v>
       </c>
       <c r="C77">
         <v>1</v>
@@ -2178,8 +2185,8 @@
       <c r="A78" s="1">
         <v>76</v>
       </c>
-      <c r="B78" t="s">
-        <v>14</v>
+      <c r="B78" s="9" t="s">
+        <v>19</v>
       </c>
       <c r="C78">
         <v>1</v>
@@ -2199,8 +2206,8 @@
       <c r="A79" s="1">
         <v>77</v>
       </c>
-      <c r="B79" t="s">
-        <v>16</v>
+      <c r="B79" s="9" t="s">
+        <v>21</v>
       </c>
       <c r="C79">
         <v>2</v>
@@ -2220,8 +2227,8 @@
       <c r="A80" s="1">
         <v>78</v>
       </c>
-      <c r="B80" t="s">
-        <v>14</v>
+      <c r="B80" s="9" t="s">
+        <v>19</v>
       </c>
       <c r="C80">
         <v>1</v>
@@ -2241,8 +2248,8 @@
       <c r="A81" s="1">
         <v>79</v>
       </c>
-      <c r="B81" t="s">
-        <v>11</v>
+      <c r="B81" s="9" t="s">
+        <v>16</v>
       </c>
       <c r="C81">
         <v>1</v>
@@ -2262,8 +2269,8 @@
       <c r="A82" s="1">
         <v>80</v>
       </c>
-      <c r="B82" t="s">
-        <v>16</v>
+      <c r="B82" s="9" t="s">
+        <v>21</v>
       </c>
       <c r="C82">
         <v>2</v>

</xml_diff>

<commit_message>
corrected typo in condition assignment sheet randomisation and output
</commit_message>
<xml_diff>
--- a/method/study 1/organiser/Study 1 Condition Assignment Sheet.xlsx
+++ b/method/study 1/organiser/Study 1 Condition Assignment Sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Ian/git/ironic-effect-of-thought-suppression-replication/method/study 1/organiser/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BFDA3AD-E18E-7B46-A6AB-D4C5DA067147}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6391242C-9542-FA48-ADAE-7FD3C299618A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="33660" windowHeight="19600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="testdata" sheetId="1" r:id="rId1"/>
@@ -144,28 +144,28 @@
     <t>random 1-2. 1 = "try NOT", 2 = "try".</t>
   </si>
   <si>
-    <t>Versuchen Sie bei Ihrer ersten Aufgabe, in den nächsten fünf Minuten an einen BERG zu denken. Ich bin in fünf Minuten zurück.</t>
+    <t>Versuchen Sie bei Ihrer ersten Aufgabe in den nächsten fünf Minuten an einen BERG zu denken. Ich bin in fünf Minuten zurück.</t>
   </si>
   <si>
-    <t>Versuchen Sie bei Ihrer ersten Aufgabe, in den nächsten fünf Minuten an ein KIND zu denken. Ich bin in fünf Minuten zurück.</t>
+    <t>Versuchen Sie bei Ihrer ersten Aufgabe in den nächsten fünf Minuten an ein KIND zu denken. Ich bin in fünf Minuten zurück.</t>
   </si>
   <si>
-    <t>Versuchen Sie bei Ihrer ersten Aufgabe, in den nächsten fünf Minuten NICHT an ein KIND zu denken. Ich bin in fünf Minuten zurück.</t>
+    <t>Versuchen Sie bei Ihrer ersten Aufgabe in den nächsten fünf Minuten NICHT an ein KIND zu denken. Ich bin in fünf Minuten zurück.</t>
   </si>
   <si>
-    <t>Versuchen Sie bei Ihrer ersten Aufgabe, in den nächsten fünf Minuten an ein HAUS zu denken. Ich bin in fünf Minuten zurück.</t>
+    <t>Versuchen Sie bei Ihrer ersten Aufgabe in den nächsten fünf Minuten an ein HAUS zu denken. Ich bin in fünf Minuten zurück.</t>
   </si>
   <si>
-    <t>Versuchen Sie bei Ihrer ersten Aufgabe, in den nächsten fünf Minuten NICHT an ein AUTO zu denken. Ich bin in fünf Minuten zurück.</t>
+    <t>Versuchen Sie bei Ihrer ersten Aufgabe in den nächsten fünf Minuten NICHT an ein AUTO zu denken. Ich bin in fünf Minuten zurück.</t>
   </si>
   <si>
-    <t>Versuchen Sie bei Ihrer ersten Aufgabe, in den nächsten fünf Minuten NICHT an ein HAUS zu denken. Ich bin in fünf Minuten zurück.</t>
+    <t>Versuchen Sie bei Ihrer ersten Aufgabe in den nächsten fünf Minuten NICHT an ein HAUS zu denken. Ich bin in fünf Minuten zurück.</t>
   </si>
   <si>
-    <t>Versuchen Sie bei Ihrer ersten Aufgabe, in den nächsten fünf Minuten NICHT an einen BERG zu denken. Ich bin in fünf Minuten zurück.</t>
+    <t>Versuchen Sie bei Ihrer ersten Aufgabe in den nächsten fünf Minuten NICHT an einen BERG zu denken. Ich bin in fünf Minuten zurück.</t>
   </si>
   <si>
-    <t>Versuchen Sie bei Ihrer ersten Aufgabe, in den nächsten fünf Minuten an ein AUTO zu denken. Ich bin in fünf Minuten zurück.</t>
+    <t>Versuchen Sie bei Ihrer ersten Aufgabe in den nächsten fünf Minuten an ein AUTO zu denken. Ich bin in fünf Minuten zurück.</t>
   </si>
 </sst>
 </file>
@@ -606,380 +606,380 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A3" s="5">
         <v>1</v>
       </c>
       <c r="B3" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C3">
-        <v>2</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="F3">
+      <c r="C3" s="9">
+        <v>2</v>
+      </c>
+      <c r="D3" s="9">
+        <v>1</v>
+      </c>
+      <c r="E3" s="9">
+        <v>1</v>
+      </c>
+      <c r="F3" s="9">
         <v>1</v>
       </c>
       <c r="G3" s="7"/>
     </row>
-    <row r="4" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A4" s="5">
         <v>2</v>
       </c>
       <c r="B4" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C4">
-        <v>2</v>
-      </c>
-      <c r="D4">
+      <c r="C4" s="9">
+        <v>2</v>
+      </c>
+      <c r="D4" s="9">
         <v>3</v>
       </c>
-      <c r="E4">
-        <v>2</v>
-      </c>
-      <c r="F4">
+      <c r="E4" s="9">
+        <v>2</v>
+      </c>
+      <c r="F4" s="9">
         <v>1</v>
       </c>
       <c r="G4" s="7"/>
     </row>
-    <row r="5" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A5" s="5">
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5">
+      <c r="C5" s="9">
+        <v>1</v>
+      </c>
+      <c r="D5" s="9">
         <v>3</v>
       </c>
-      <c r="E5">
-        <v>2</v>
-      </c>
-      <c r="F5">
+      <c r="E5" s="9">
+        <v>2</v>
+      </c>
+      <c r="F5" s="9">
         <v>1</v>
       </c>
       <c r="G5" s="7"/>
     </row>
-    <row r="6" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A6" s="5">
         <v>4</v>
       </c>
       <c r="B6" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C6">
-        <v>2</v>
-      </c>
-      <c r="D6">
+      <c r="C6" s="9">
+        <v>2</v>
+      </c>
+      <c r="D6" s="9">
         <v>4</v>
       </c>
-      <c r="E6">
-        <v>2</v>
-      </c>
-      <c r="F6">
+      <c r="E6" s="9">
+        <v>2</v>
+      </c>
+      <c r="F6" s="9">
         <v>2</v>
       </c>
       <c r="G6" s="7"/>
     </row>
-    <row r="7" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A7" s="5">
         <v>5</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C7">
-        <v>1</v>
-      </c>
-      <c r="D7">
-        <v>2</v>
-      </c>
-      <c r="E7">
-        <v>1</v>
-      </c>
-      <c r="F7">
+      <c r="C7" s="9">
+        <v>1</v>
+      </c>
+      <c r="D7" s="9">
+        <v>2</v>
+      </c>
+      <c r="E7" s="9">
+        <v>1</v>
+      </c>
+      <c r="F7" s="9">
         <v>2</v>
       </c>
       <c r="G7" s="7"/>
     </row>
-    <row r="8" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A8" s="5">
         <v>6</v>
       </c>
       <c r="B8" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C8">
-        <v>2</v>
-      </c>
-      <c r="D8">
+      <c r="C8" s="9">
+        <v>2</v>
+      </c>
+      <c r="D8" s="9">
         <v>4</v>
       </c>
-      <c r="E8">
-        <v>2</v>
-      </c>
-      <c r="F8">
+      <c r="E8" s="9">
+        <v>2</v>
+      </c>
+      <c r="F8" s="9">
         <v>2</v>
       </c>
       <c r="G8" s="7"/>
     </row>
-    <row r="9" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A9" s="5">
         <v>7</v>
       </c>
       <c r="B9" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C9">
-        <v>2</v>
-      </c>
-      <c r="D9">
-        <v>1</v>
-      </c>
-      <c r="E9">
-        <v>1</v>
-      </c>
-      <c r="F9">
+      <c r="C9" s="9">
+        <v>2</v>
+      </c>
+      <c r="D9" s="9">
+        <v>1</v>
+      </c>
+      <c r="E9" s="9">
+        <v>1</v>
+      </c>
+      <c r="F9" s="9">
         <v>1</v>
       </c>
       <c r="G9" s="7"/>
     </row>
-    <row r="10" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A10" s="5">
         <v>8</v>
       </c>
       <c r="B10" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C10">
-        <v>1</v>
-      </c>
-      <c r="D10">
+      <c r="C10" s="9">
+        <v>1</v>
+      </c>
+      <c r="D10" s="9">
         <v>3</v>
       </c>
-      <c r="E10">
-        <v>2</v>
-      </c>
-      <c r="F10">
+      <c r="E10" s="9">
+        <v>2</v>
+      </c>
+      <c r="F10" s="9">
         <v>2</v>
       </c>
       <c r="G10" s="7"/>
     </row>
-    <row r="11" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A11" s="5">
         <v>9</v>
       </c>
       <c r="B11" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C11">
-        <v>2</v>
-      </c>
-      <c r="D11">
+      <c r="C11" s="9">
+        <v>2</v>
+      </c>
+      <c r="D11" s="9">
         <v>4</v>
       </c>
-      <c r="E11">
-        <v>2</v>
-      </c>
-      <c r="F11">
+      <c r="E11" s="9">
+        <v>2</v>
+      </c>
+      <c r="F11" s="9">
         <v>1</v>
       </c>
       <c r="G11" s="7"/>
     </row>
-    <row r="12" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A12" s="5">
         <v>10</v>
       </c>
       <c r="B12" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C12">
-        <v>1</v>
-      </c>
-      <c r="D12">
+      <c r="C12" s="9">
+        <v>1</v>
+      </c>
+      <c r="D12" s="9">
         <v>4</v>
       </c>
-      <c r="E12">
-        <v>2</v>
-      </c>
-      <c r="F12">
+      <c r="E12" s="9">
+        <v>2</v>
+      </c>
+      <c r="F12" s="9">
         <v>1</v>
       </c>
       <c r="G12" s="7"/>
     </row>
-    <row r="13" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A13" s="5">
         <v>11</v>
       </c>
       <c r="B13" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C13">
-        <v>1</v>
-      </c>
-      <c r="D13">
-        <v>2</v>
-      </c>
-      <c r="E13">
-        <v>1</v>
-      </c>
-      <c r="F13">
+      <c r="C13" s="9">
+        <v>1</v>
+      </c>
+      <c r="D13" s="9">
+        <v>2</v>
+      </c>
+      <c r="E13" s="9">
+        <v>1</v>
+      </c>
+      <c r="F13" s="9">
         <v>2</v>
       </c>
       <c r="G13" s="7"/>
     </row>
-    <row r="14" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A14" s="5">
         <v>12</v>
       </c>
       <c r="B14" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C14">
-        <v>1</v>
-      </c>
-      <c r="D14">
+      <c r="C14" s="9">
+        <v>1</v>
+      </c>
+      <c r="D14" s="9">
         <v>3</v>
       </c>
-      <c r="E14">
-        <v>2</v>
-      </c>
-      <c r="F14">
+      <c r="E14" s="9">
+        <v>2</v>
+      </c>
+      <c r="F14" s="9">
         <v>2</v>
       </c>
       <c r="G14" s="7"/>
     </row>
-    <row r="15" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A15" s="5">
         <v>13</v>
       </c>
       <c r="B15" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C15">
-        <v>1</v>
-      </c>
-      <c r="D15">
-        <v>1</v>
-      </c>
-      <c r="E15">
-        <v>1</v>
-      </c>
-      <c r="F15">
+      <c r="C15" s="9">
+        <v>1</v>
+      </c>
+      <c r="D15" s="9">
+        <v>1</v>
+      </c>
+      <c r="E15" s="9">
+        <v>1</v>
+      </c>
+      <c r="F15" s="9">
         <v>1</v>
       </c>
       <c r="G15" s="7"/>
     </row>
-    <row r="16" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A16" s="5">
         <v>14</v>
       </c>
       <c r="B16" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C16">
-        <v>2</v>
-      </c>
-      <c r="D16">
-        <v>1</v>
-      </c>
-      <c r="E16">
-        <v>1</v>
-      </c>
-      <c r="F16">
+      <c r="C16" s="9">
+        <v>2</v>
+      </c>
+      <c r="D16" s="9">
+        <v>1</v>
+      </c>
+      <c r="E16" s="9">
+        <v>1</v>
+      </c>
+      <c r="F16" s="9">
         <v>1</v>
       </c>
       <c r="G16" s="7"/>
     </row>
-    <row r="17" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A17" s="5">
         <v>15</v>
       </c>
       <c r="B17" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C17">
-        <v>1</v>
-      </c>
-      <c r="D17">
+      <c r="C17" s="9">
+        <v>1</v>
+      </c>
+      <c r="D17" s="9">
         <v>3</v>
       </c>
-      <c r="E17">
-        <v>2</v>
-      </c>
-      <c r="F17">
+      <c r="E17" s="9">
+        <v>2</v>
+      </c>
+      <c r="F17" s="9">
         <v>1</v>
       </c>
       <c r="G17" s="7"/>
     </row>
-    <row r="18" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A18" s="5">
         <v>16</v>
       </c>
       <c r="B18" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C18">
-        <v>1</v>
-      </c>
-      <c r="D18">
+      <c r="C18" s="9">
+        <v>1</v>
+      </c>
+      <c r="D18" s="9">
         <v>4</v>
       </c>
-      <c r="E18">
-        <v>2</v>
-      </c>
-      <c r="F18">
+      <c r="E18" s="9">
+        <v>2</v>
+      </c>
+      <c r="F18" s="9">
         <v>2</v>
       </c>
       <c r="G18" s="7"/>
     </row>
-    <row r="19" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A19" s="5">
         <v>17</v>
       </c>
       <c r="B19" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C19">
-        <v>2</v>
-      </c>
-      <c r="D19">
+      <c r="C19" s="9">
+        <v>2</v>
+      </c>
+      <c r="D19" s="9">
         <v>4</v>
       </c>
-      <c r="E19">
-        <v>2</v>
-      </c>
-      <c r="F19">
+      <c r="E19" s="9">
+        <v>2</v>
+      </c>
+      <c r="F19" s="9">
         <v>2</v>
       </c>
       <c r="G19" s="7"/>
     </row>
-    <row r="20" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A20" s="5">
         <v>18</v>
       </c>
       <c r="B20" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C20">
-        <v>1</v>
-      </c>
-      <c r="D20">
+      <c r="C20" s="9">
+        <v>1</v>
+      </c>
+      <c r="D20" s="9">
         <v>4</v>
       </c>
-      <c r="E20">
-        <v>2</v>
-      </c>
-      <c r="F20">
+      <c r="E20" s="9">
+        <v>2</v>
+      </c>
+      <c r="F20" s="9">
         <v>1</v>
       </c>
       <c r="G20" s="7"/>
@@ -991,16 +991,16 @@
       <c r="B21" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C21">
-        <v>2</v>
-      </c>
-      <c r="D21">
-        <v>1</v>
-      </c>
-      <c r="E21">
-        <v>1</v>
-      </c>
-      <c r="F21">
+      <c r="C21" s="9">
+        <v>2</v>
+      </c>
+      <c r="D21" s="9">
+        <v>1</v>
+      </c>
+      <c r="E21" s="9">
+        <v>1</v>
+      </c>
+      <c r="F21" s="9">
         <v>1</v>
       </c>
       <c r="G21" s="8"/>
@@ -1012,16 +1012,16 @@
       <c r="B22" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C22">
-        <v>1</v>
-      </c>
-      <c r="D22">
-        <v>1</v>
-      </c>
-      <c r="E22">
-        <v>1</v>
-      </c>
-      <c r="F22">
+      <c r="C22" s="9">
+        <v>1</v>
+      </c>
+      <c r="D22" s="9">
+        <v>1</v>
+      </c>
+      <c r="E22" s="9">
+        <v>1</v>
+      </c>
+      <c r="F22" s="9">
         <v>1</v>
       </c>
       <c r="G22" s="8"/>
@@ -1033,16 +1033,16 @@
       <c r="B23" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C23">
-        <v>2</v>
-      </c>
-      <c r="D23">
+      <c r="C23" s="9">
+        <v>2</v>
+      </c>
+      <c r="D23" s="9">
         <v>3</v>
       </c>
-      <c r="E23">
-        <v>2</v>
-      </c>
-      <c r="F23">
+      <c r="E23" s="9">
+        <v>2</v>
+      </c>
+      <c r="F23" s="9">
         <v>2</v>
       </c>
       <c r="G23" s="8"/>
@@ -1054,16 +1054,16 @@
       <c r="B24" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C24">
-        <v>1</v>
-      </c>
-      <c r="D24">
+      <c r="C24" s="9">
+        <v>1</v>
+      </c>
+      <c r="D24" s="9">
         <v>4</v>
       </c>
-      <c r="E24">
-        <v>2</v>
-      </c>
-      <c r="F24">
+      <c r="E24" s="9">
+        <v>2</v>
+      </c>
+      <c r="F24" s="9">
         <v>2</v>
       </c>
       <c r="G24" s="8"/>
@@ -1075,16 +1075,16 @@
       <c r="B25" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C25">
-        <v>1</v>
-      </c>
-      <c r="D25">
+      <c r="C25" s="9">
+        <v>1</v>
+      </c>
+      <c r="D25" s="9">
         <v>3</v>
       </c>
-      <c r="E25">
-        <v>2</v>
-      </c>
-      <c r="F25">
+      <c r="E25" s="9">
+        <v>2</v>
+      </c>
+      <c r="F25" s="9">
         <v>2</v>
       </c>
       <c r="G25" s="8"/>
@@ -1096,16 +1096,16 @@
       <c r="B26" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C26">
-        <v>1</v>
-      </c>
-      <c r="D26">
+      <c r="C26" s="9">
+        <v>1</v>
+      </c>
+      <c r="D26" s="9">
         <v>4</v>
       </c>
-      <c r="E26">
-        <v>2</v>
-      </c>
-      <c r="F26">
+      <c r="E26" s="9">
+        <v>2</v>
+      </c>
+      <c r="F26" s="9">
         <v>2</v>
       </c>
       <c r="G26" s="8"/>
@@ -1117,16 +1117,16 @@
       <c r="B27" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C27">
-        <v>2</v>
-      </c>
-      <c r="D27">
+      <c r="C27" s="9">
+        <v>2</v>
+      </c>
+      <c r="D27" s="9">
         <v>3</v>
       </c>
-      <c r="E27">
-        <v>2</v>
-      </c>
-      <c r="F27">
+      <c r="E27" s="9">
+        <v>2</v>
+      </c>
+      <c r="F27" s="9">
         <v>2</v>
       </c>
       <c r="G27" s="8"/>
@@ -1138,16 +1138,16 @@
       <c r="B28" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C28">
-        <v>1</v>
-      </c>
-      <c r="D28">
+      <c r="C28" s="9">
+        <v>1</v>
+      </c>
+      <c r="D28" s="9">
         <v>4</v>
       </c>
-      <c r="E28">
-        <v>2</v>
-      </c>
-      <c r="F28">
+      <c r="E28" s="9">
+        <v>2</v>
+      </c>
+      <c r="F28" s="9">
         <v>1</v>
       </c>
       <c r="G28" s="8"/>
@@ -1159,16 +1159,16 @@
       <c r="B29" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C29">
-        <v>2</v>
-      </c>
-      <c r="D29">
-        <v>1</v>
-      </c>
-      <c r="E29">
-        <v>1</v>
-      </c>
-      <c r="F29">
+      <c r="C29" s="9">
+        <v>2</v>
+      </c>
+      <c r="D29" s="9">
+        <v>1</v>
+      </c>
+      <c r="E29" s="9">
+        <v>1</v>
+      </c>
+      <c r="F29" s="9">
         <v>2</v>
       </c>
       <c r="G29" s="8"/>
@@ -1180,16 +1180,16 @@
       <c r="B30" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C30">
-        <v>2</v>
-      </c>
-      <c r="D30">
+      <c r="C30" s="9">
+        <v>2</v>
+      </c>
+      <c r="D30" s="9">
         <v>4</v>
       </c>
-      <c r="E30">
-        <v>2</v>
-      </c>
-      <c r="F30">
+      <c r="E30" s="9">
+        <v>2</v>
+      </c>
+      <c r="F30" s="9">
         <v>1</v>
       </c>
       <c r="G30" s="8"/>
@@ -1201,16 +1201,16 @@
       <c r="B31" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C31">
-        <v>1</v>
-      </c>
-      <c r="D31">
+      <c r="C31" s="9">
+        <v>1</v>
+      </c>
+      <c r="D31" s="9">
         <v>3</v>
       </c>
-      <c r="E31">
-        <v>2</v>
-      </c>
-      <c r="F31">
+      <c r="E31" s="9">
+        <v>2</v>
+      </c>
+      <c r="F31" s="9">
         <v>2</v>
       </c>
       <c r="G31" s="8"/>
@@ -1222,16 +1222,16 @@
       <c r="B32" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C32">
-        <v>2</v>
-      </c>
-      <c r="D32">
-        <v>1</v>
-      </c>
-      <c r="E32">
-        <v>1</v>
-      </c>
-      <c r="F32">
+      <c r="C32" s="9">
+        <v>2</v>
+      </c>
+      <c r="D32" s="9">
+        <v>1</v>
+      </c>
+      <c r="E32" s="9">
+        <v>1</v>
+      </c>
+      <c r="F32" s="9">
         <v>1</v>
       </c>
       <c r="G32" s="8"/>
@@ -1243,16 +1243,16 @@
       <c r="B33" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C33">
-        <v>1</v>
-      </c>
-      <c r="D33">
-        <v>2</v>
-      </c>
-      <c r="E33">
-        <v>1</v>
-      </c>
-      <c r="F33">
+      <c r="C33" s="9">
+        <v>1</v>
+      </c>
+      <c r="D33" s="9">
+        <v>2</v>
+      </c>
+      <c r="E33" s="9">
+        <v>1</v>
+      </c>
+      <c r="F33" s="9">
         <v>1</v>
       </c>
       <c r="G33" s="8"/>
@@ -1264,16 +1264,16 @@
       <c r="B34" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C34">
-        <v>1</v>
-      </c>
-      <c r="D34">
+      <c r="C34" s="9">
+        <v>1</v>
+      </c>
+      <c r="D34" s="9">
         <v>3</v>
       </c>
-      <c r="E34">
-        <v>2</v>
-      </c>
-      <c r="F34">
+      <c r="E34" s="9">
+        <v>2</v>
+      </c>
+      <c r="F34" s="9">
         <v>2</v>
       </c>
       <c r="G34" s="8"/>
@@ -1285,16 +1285,16 @@
       <c r="B35" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C35">
-        <v>1</v>
-      </c>
-      <c r="D35">
-        <v>1</v>
-      </c>
-      <c r="E35">
-        <v>1</v>
-      </c>
-      <c r="F35">
+      <c r="C35" s="9">
+        <v>1</v>
+      </c>
+      <c r="D35" s="9">
+        <v>1</v>
+      </c>
+      <c r="E35" s="9">
+        <v>1</v>
+      </c>
+      <c r="F35" s="9">
         <v>2</v>
       </c>
       <c r="G35" s="8"/>
@@ -1306,16 +1306,16 @@
       <c r="B36" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C36">
-        <v>2</v>
-      </c>
-      <c r="D36">
+      <c r="C36" s="9">
+        <v>2</v>
+      </c>
+      <c r="D36" s="9">
         <v>4</v>
       </c>
-      <c r="E36">
-        <v>2</v>
-      </c>
-      <c r="F36">
+      <c r="E36" s="9">
+        <v>2</v>
+      </c>
+      <c r="F36" s="9">
         <v>1</v>
       </c>
       <c r="G36" s="8"/>
@@ -1327,16 +1327,16 @@
       <c r="B37" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C37">
-        <v>1</v>
-      </c>
-      <c r="D37">
-        <v>1</v>
-      </c>
-      <c r="E37">
-        <v>1</v>
-      </c>
-      <c r="F37">
+      <c r="C37" s="9">
+        <v>1</v>
+      </c>
+      <c r="D37" s="9">
+        <v>1</v>
+      </c>
+      <c r="E37" s="9">
+        <v>1</v>
+      </c>
+      <c r="F37" s="9">
         <v>2</v>
       </c>
       <c r="G37" s="8"/>
@@ -1348,16 +1348,16 @@
       <c r="B38" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C38">
-        <v>2</v>
-      </c>
-      <c r="D38">
+      <c r="C38" s="9">
+        <v>2</v>
+      </c>
+      <c r="D38" s="9">
         <v>4</v>
       </c>
-      <c r="E38">
-        <v>2</v>
-      </c>
-      <c r="F38">
+      <c r="E38" s="9">
+        <v>2</v>
+      </c>
+      <c r="F38" s="9">
         <v>1</v>
       </c>
       <c r="G38" s="8"/>
@@ -1369,16 +1369,16 @@
       <c r="B39" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C39">
-        <v>2</v>
-      </c>
-      <c r="D39">
+      <c r="C39" s="9">
+        <v>2</v>
+      </c>
+      <c r="D39" s="9">
         <v>4</v>
       </c>
-      <c r="E39">
-        <v>2</v>
-      </c>
-      <c r="F39">
+      <c r="E39" s="9">
+        <v>2</v>
+      </c>
+      <c r="F39" s="9">
         <v>2</v>
       </c>
       <c r="G39" s="8"/>
@@ -1390,16 +1390,16 @@
       <c r="B40" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C40">
-        <v>2</v>
-      </c>
-      <c r="D40">
-        <v>2</v>
-      </c>
-      <c r="E40">
-        <v>1</v>
-      </c>
-      <c r="F40">
+      <c r="C40" s="9">
+        <v>2</v>
+      </c>
+      <c r="D40" s="9">
+        <v>2</v>
+      </c>
+      <c r="E40" s="9">
+        <v>1</v>
+      </c>
+      <c r="F40" s="9">
         <v>2</v>
       </c>
       <c r="G40" s="8"/>
@@ -1411,16 +1411,16 @@
       <c r="B41" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C41">
-        <v>2</v>
-      </c>
-      <c r="D41">
+      <c r="C41" s="9">
+        <v>2</v>
+      </c>
+      <c r="D41" s="9">
         <v>3</v>
       </c>
-      <c r="E41">
-        <v>2</v>
-      </c>
-      <c r="F41">
+      <c r="E41" s="9">
+        <v>2</v>
+      </c>
+      <c r="F41" s="9">
         <v>1</v>
       </c>
       <c r="G41" s="8"/>
@@ -1432,16 +1432,16 @@
       <c r="B42" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C42">
-        <v>2</v>
-      </c>
-      <c r="D42">
-        <v>1</v>
-      </c>
-      <c r="E42">
-        <v>1</v>
-      </c>
-      <c r="F42">
+      <c r="C42" s="9">
+        <v>2</v>
+      </c>
+      <c r="D42" s="9">
+        <v>1</v>
+      </c>
+      <c r="E42" s="9">
+        <v>1</v>
+      </c>
+      <c r="F42" s="9">
         <v>2</v>
       </c>
       <c r="G42" s="8"/>
@@ -1453,16 +1453,16 @@
       <c r="B43" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C43">
-        <v>2</v>
-      </c>
-      <c r="D43">
-        <v>2</v>
-      </c>
-      <c r="E43">
-        <v>1</v>
-      </c>
-      <c r="F43">
+      <c r="C43" s="9">
+        <v>2</v>
+      </c>
+      <c r="D43" s="9">
+        <v>2</v>
+      </c>
+      <c r="E43" s="9">
+        <v>1</v>
+      </c>
+      <c r="F43" s="9">
         <v>1</v>
       </c>
       <c r="G43" s="8"/>
@@ -1474,16 +1474,16 @@
       <c r="B44" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C44">
-        <v>1</v>
-      </c>
-      <c r="D44">
+      <c r="C44" s="9">
+        <v>1</v>
+      </c>
+      <c r="D44" s="9">
         <v>4</v>
       </c>
-      <c r="E44">
-        <v>2</v>
-      </c>
-      <c r="F44">
+      <c r="E44" s="9">
+        <v>2</v>
+      </c>
+      <c r="F44" s="9">
         <v>1</v>
       </c>
       <c r="G44" s="8"/>
@@ -1495,16 +1495,16 @@
       <c r="B45" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C45">
-        <v>2</v>
-      </c>
-      <c r="D45">
-        <v>2</v>
-      </c>
-      <c r="E45">
-        <v>1</v>
-      </c>
-      <c r="F45">
+      <c r="C45" s="9">
+        <v>2</v>
+      </c>
+      <c r="D45" s="9">
+        <v>2</v>
+      </c>
+      <c r="E45" s="9">
+        <v>1</v>
+      </c>
+      <c r="F45" s="9">
         <v>1</v>
       </c>
       <c r="G45" s="8"/>
@@ -1516,16 +1516,16 @@
       <c r="B46" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C46">
-        <v>1</v>
-      </c>
-      <c r="D46">
+      <c r="C46" s="9">
+        <v>1</v>
+      </c>
+      <c r="D46" s="9">
         <v>3</v>
       </c>
-      <c r="E46">
-        <v>2</v>
-      </c>
-      <c r="F46">
+      <c r="E46" s="9">
+        <v>2</v>
+      </c>
+      <c r="F46" s="9">
         <v>1</v>
       </c>
       <c r="G46" s="8"/>
@@ -1537,16 +1537,16 @@
       <c r="B47" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C47">
-        <v>2</v>
-      </c>
-      <c r="D47">
+      <c r="C47" s="9">
+        <v>2</v>
+      </c>
+      <c r="D47" s="9">
         <v>3</v>
       </c>
-      <c r="E47">
-        <v>2</v>
-      </c>
-      <c r="F47">
+      <c r="E47" s="9">
+        <v>2</v>
+      </c>
+      <c r="F47" s="9">
         <v>1</v>
       </c>
       <c r="G47" s="8"/>
@@ -1558,16 +1558,16 @@
       <c r="B48" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C48">
-        <v>1</v>
-      </c>
-      <c r="D48">
-        <v>1</v>
-      </c>
-      <c r="E48">
-        <v>1</v>
-      </c>
-      <c r="F48">
+      <c r="C48" s="9">
+        <v>1</v>
+      </c>
+      <c r="D48" s="9">
+        <v>1</v>
+      </c>
+      <c r="E48" s="9">
+        <v>1</v>
+      </c>
+      <c r="F48" s="9">
         <v>2</v>
       </c>
       <c r="G48" s="8"/>
@@ -1579,16 +1579,16 @@
       <c r="B49" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C49">
-        <v>1</v>
-      </c>
-      <c r="D49">
+      <c r="C49" s="9">
+        <v>1</v>
+      </c>
+      <c r="D49" s="9">
         <v>4</v>
       </c>
-      <c r="E49">
-        <v>2</v>
-      </c>
-      <c r="F49">
+      <c r="E49" s="9">
+        <v>2</v>
+      </c>
+      <c r="F49" s="9">
         <v>1</v>
       </c>
       <c r="G49" s="8"/>
@@ -1600,16 +1600,16 @@
       <c r="B50" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C50">
-        <v>1</v>
-      </c>
-      <c r="D50">
-        <v>1</v>
-      </c>
-      <c r="E50">
-        <v>1</v>
-      </c>
-      <c r="F50">
+      <c r="C50" s="9">
+        <v>1</v>
+      </c>
+      <c r="D50" s="9">
+        <v>1</v>
+      </c>
+      <c r="E50" s="9">
+        <v>1</v>
+      </c>
+      <c r="F50" s="9">
         <v>2</v>
       </c>
       <c r="G50" s="8"/>
@@ -1621,16 +1621,16 @@
       <c r="B51" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C51">
-        <v>2</v>
-      </c>
-      <c r="D51">
-        <v>2</v>
-      </c>
-      <c r="E51">
-        <v>1</v>
-      </c>
-      <c r="F51">
+      <c r="C51" s="9">
+        <v>2</v>
+      </c>
+      <c r="D51" s="9">
+        <v>2</v>
+      </c>
+      <c r="E51" s="9">
+        <v>1</v>
+      </c>
+      <c r="F51" s="9">
         <v>2</v>
       </c>
       <c r="G51" s="8"/>
@@ -1642,16 +1642,16 @@
       <c r="B52" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C52">
-        <v>2</v>
-      </c>
-      <c r="D52">
-        <v>2</v>
-      </c>
-      <c r="E52">
-        <v>1</v>
-      </c>
-      <c r="F52">
+      <c r="C52" s="9">
+        <v>2</v>
+      </c>
+      <c r="D52" s="9">
+        <v>2</v>
+      </c>
+      <c r="E52" s="9">
+        <v>1</v>
+      </c>
+      <c r="F52" s="9">
         <v>2</v>
       </c>
       <c r="G52" s="8"/>
@@ -1663,16 +1663,16 @@
       <c r="B53" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C53">
-        <v>2</v>
-      </c>
-      <c r="D53">
+      <c r="C53" s="9">
+        <v>2</v>
+      </c>
+      <c r="D53" s="9">
         <v>3</v>
       </c>
-      <c r="E53">
-        <v>2</v>
-      </c>
-      <c r="F53">
+      <c r="E53" s="9">
+        <v>2</v>
+      </c>
+      <c r="F53" s="9">
         <v>2</v>
       </c>
       <c r="G53" s="8"/>
@@ -1684,16 +1684,16 @@
       <c r="B54" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C54">
-        <v>1</v>
-      </c>
-      <c r="D54">
+      <c r="C54" s="9">
+        <v>1</v>
+      </c>
+      <c r="D54" s="9">
         <v>3</v>
       </c>
-      <c r="E54">
-        <v>2</v>
-      </c>
-      <c r="F54">
+      <c r="E54" s="9">
+        <v>2</v>
+      </c>
+      <c r="F54" s="9">
         <v>1</v>
       </c>
       <c r="G54" s="8"/>
@@ -1705,16 +1705,16 @@
       <c r="B55" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C55">
-        <v>2</v>
-      </c>
-      <c r="D55">
-        <v>2</v>
-      </c>
-      <c r="E55">
-        <v>1</v>
-      </c>
-      <c r="F55">
+      <c r="C55" s="9">
+        <v>2</v>
+      </c>
+      <c r="D55" s="9">
+        <v>2</v>
+      </c>
+      <c r="E55" s="9">
+        <v>1</v>
+      </c>
+      <c r="F55" s="9">
         <v>1</v>
       </c>
       <c r="G55" s="8"/>
@@ -1726,16 +1726,16 @@
       <c r="B56" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C56">
-        <v>2</v>
-      </c>
-      <c r="D56">
+      <c r="C56" s="9">
+        <v>2</v>
+      </c>
+      <c r="D56" s="9">
         <v>3</v>
       </c>
-      <c r="E56">
-        <v>2</v>
-      </c>
-      <c r="F56">
+      <c r="E56" s="9">
+        <v>2</v>
+      </c>
+      <c r="F56" s="9">
         <v>2</v>
       </c>
       <c r="G56" s="8"/>
@@ -1747,16 +1747,16 @@
       <c r="B57" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C57">
-        <v>2</v>
-      </c>
-      <c r="D57">
-        <v>2</v>
-      </c>
-      <c r="E57">
-        <v>1</v>
-      </c>
-      <c r="F57">
+      <c r="C57" s="9">
+        <v>2</v>
+      </c>
+      <c r="D57" s="9">
+        <v>2</v>
+      </c>
+      <c r="E57" s="9">
+        <v>1</v>
+      </c>
+      <c r="F57" s="9">
         <v>1</v>
       </c>
       <c r="G57" s="8"/>
@@ -1768,16 +1768,16 @@
       <c r="B58" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C58">
-        <v>1</v>
-      </c>
-      <c r="D58">
-        <v>1</v>
-      </c>
-      <c r="E58">
-        <v>1</v>
-      </c>
-      <c r="F58">
+      <c r="C58" s="9">
+        <v>1</v>
+      </c>
+      <c r="D58" s="9">
+        <v>1</v>
+      </c>
+      <c r="E58" s="9">
+        <v>1</v>
+      </c>
+      <c r="F58" s="9">
         <v>2</v>
       </c>
       <c r="G58" s="8"/>
@@ -1789,16 +1789,16 @@
       <c r="B59" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C59">
-        <v>2</v>
-      </c>
-      <c r="D59">
-        <v>1</v>
-      </c>
-      <c r="E59">
-        <v>1</v>
-      </c>
-      <c r="F59">
+      <c r="C59" s="9">
+        <v>2</v>
+      </c>
+      <c r="D59" s="9">
+        <v>1</v>
+      </c>
+      <c r="E59" s="9">
+        <v>1</v>
+      </c>
+      <c r="F59" s="9">
         <v>2</v>
       </c>
       <c r="G59" s="8"/>
@@ -1810,16 +1810,16 @@
       <c r="B60" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C60">
-        <v>2</v>
-      </c>
-      <c r="D60">
-        <v>2</v>
-      </c>
-      <c r="E60">
-        <v>1</v>
-      </c>
-      <c r="F60">
+      <c r="C60" s="9">
+        <v>2</v>
+      </c>
+      <c r="D60" s="9">
+        <v>2</v>
+      </c>
+      <c r="E60" s="9">
+        <v>1</v>
+      </c>
+      <c r="F60" s="9">
         <v>2</v>
       </c>
       <c r="G60" s="8"/>
@@ -1831,16 +1831,16 @@
       <c r="B61" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C61">
-        <v>1</v>
-      </c>
-      <c r="D61">
-        <v>1</v>
-      </c>
-      <c r="E61">
-        <v>1</v>
-      </c>
-      <c r="F61">
+      <c r="C61" s="9">
+        <v>1</v>
+      </c>
+      <c r="D61" s="9">
+        <v>1</v>
+      </c>
+      <c r="E61" s="9">
+        <v>1</v>
+      </c>
+      <c r="F61" s="9">
         <v>1</v>
       </c>
       <c r="G61" s="8"/>
@@ -1852,16 +1852,16 @@
       <c r="B62" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C62">
-        <v>1</v>
-      </c>
-      <c r="D62">
-        <v>2</v>
-      </c>
-      <c r="E62">
-        <v>1</v>
-      </c>
-      <c r="F62">
+      <c r="C62" s="9">
+        <v>1</v>
+      </c>
+      <c r="D62" s="9">
+        <v>2</v>
+      </c>
+      <c r="E62" s="9">
+        <v>1</v>
+      </c>
+      <c r="F62" s="9">
         <v>1</v>
       </c>
       <c r="G62" s="8"/>
@@ -1873,16 +1873,16 @@
       <c r="B63" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C63">
-        <v>1</v>
-      </c>
-      <c r="D63">
-        <v>1</v>
-      </c>
-      <c r="E63">
-        <v>1</v>
-      </c>
-      <c r="F63">
+      <c r="C63" s="9">
+        <v>1</v>
+      </c>
+      <c r="D63" s="9">
+        <v>1</v>
+      </c>
+      <c r="E63" s="9">
+        <v>1</v>
+      </c>
+      <c r="F63" s="9">
         <v>1</v>
       </c>
       <c r="G63" s="8"/>
@@ -1894,16 +1894,16 @@
       <c r="B64" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C64">
-        <v>2</v>
-      </c>
-      <c r="D64">
+      <c r="C64" s="9">
+        <v>2</v>
+      </c>
+      <c r="D64" s="9">
         <v>3</v>
       </c>
-      <c r="E64">
-        <v>2</v>
-      </c>
-      <c r="F64">
+      <c r="E64" s="9">
+        <v>2</v>
+      </c>
+      <c r="F64" s="9">
         <v>1</v>
       </c>
       <c r="G64" s="8"/>
@@ -1915,16 +1915,16 @@
       <c r="B65" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C65">
-        <v>1</v>
-      </c>
-      <c r="D65">
-        <v>2</v>
-      </c>
-      <c r="E65">
-        <v>1</v>
-      </c>
-      <c r="F65">
+      <c r="C65" s="9">
+        <v>1</v>
+      </c>
+      <c r="D65" s="9">
+        <v>2</v>
+      </c>
+      <c r="E65" s="9">
+        <v>1</v>
+      </c>
+      <c r="F65" s="9">
         <v>1</v>
       </c>
       <c r="G65" s="8"/>
@@ -1936,16 +1936,16 @@
       <c r="B66" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C66">
-        <v>2</v>
-      </c>
-      <c r="D66">
+      <c r="C66" s="9">
+        <v>2</v>
+      </c>
+      <c r="D66" s="9">
         <v>4</v>
       </c>
-      <c r="E66">
-        <v>2</v>
-      </c>
-      <c r="F66">
+      <c r="E66" s="9">
+        <v>2</v>
+      </c>
+      <c r="F66" s="9">
         <v>2</v>
       </c>
       <c r="G66" s="8"/>
@@ -1957,16 +1957,16 @@
       <c r="B67" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C67">
-        <v>1</v>
-      </c>
-      <c r="D67">
-        <v>1</v>
-      </c>
-      <c r="E67">
-        <v>1</v>
-      </c>
-      <c r="F67">
+      <c r="C67" s="9">
+        <v>1</v>
+      </c>
+      <c r="D67" s="9">
+        <v>1</v>
+      </c>
+      <c r="E67" s="9">
+        <v>1</v>
+      </c>
+      <c r="F67" s="9">
         <v>1</v>
       </c>
       <c r="G67" s="8"/>
@@ -1978,16 +1978,16 @@
       <c r="B68" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C68">
-        <v>2</v>
-      </c>
-      <c r="D68">
-        <v>1</v>
-      </c>
-      <c r="E68">
-        <v>1</v>
-      </c>
-      <c r="F68">
+      <c r="C68" s="9">
+        <v>2</v>
+      </c>
+      <c r="D68" s="9">
+        <v>1</v>
+      </c>
+      <c r="E68" s="9">
+        <v>1</v>
+      </c>
+      <c r="F68" s="9">
         <v>2</v>
       </c>
       <c r="G68" s="8"/>
@@ -1999,16 +1999,16 @@
       <c r="B69" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C69">
-        <v>1</v>
-      </c>
-      <c r="D69">
-        <v>2</v>
-      </c>
-      <c r="E69">
-        <v>1</v>
-      </c>
-      <c r="F69">
+      <c r="C69" s="9">
+        <v>1</v>
+      </c>
+      <c r="D69" s="9">
+        <v>2</v>
+      </c>
+      <c r="E69" s="9">
+        <v>1</v>
+      </c>
+      <c r="F69" s="9">
         <v>2</v>
       </c>
       <c r="G69" s="8"/>
@@ -2020,16 +2020,16 @@
       <c r="B70" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C70">
-        <v>1</v>
-      </c>
-      <c r="D70">
-        <v>2</v>
-      </c>
-      <c r="E70">
-        <v>1</v>
-      </c>
-      <c r="F70">
+      <c r="C70" s="9">
+        <v>1</v>
+      </c>
+      <c r="D70" s="9">
+        <v>2</v>
+      </c>
+      <c r="E70" s="9">
+        <v>1</v>
+      </c>
+      <c r="F70" s="9">
         <v>1</v>
       </c>
       <c r="G70" s="8"/>
@@ -2041,16 +2041,16 @@
       <c r="B71" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C71">
-        <v>1</v>
-      </c>
-      <c r="D71">
-        <v>2</v>
-      </c>
-      <c r="E71">
-        <v>1</v>
-      </c>
-      <c r="F71">
+      <c r="C71" s="9">
+        <v>1</v>
+      </c>
+      <c r="D71" s="9">
+        <v>2</v>
+      </c>
+      <c r="E71" s="9">
+        <v>1</v>
+      </c>
+      <c r="F71" s="9">
         <v>2</v>
       </c>
       <c r="G71" s="8"/>
@@ -2062,16 +2062,16 @@
       <c r="B72" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C72">
-        <v>1</v>
-      </c>
-      <c r="D72">
-        <v>2</v>
-      </c>
-      <c r="E72">
-        <v>1</v>
-      </c>
-      <c r="F72">
+      <c r="C72" s="9">
+        <v>1</v>
+      </c>
+      <c r="D72" s="9">
+        <v>2</v>
+      </c>
+      <c r="E72" s="9">
+        <v>1</v>
+      </c>
+      <c r="F72" s="9">
         <v>1</v>
       </c>
       <c r="G72" s="8"/>
@@ -2083,16 +2083,16 @@
       <c r="B73" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C73">
-        <v>2</v>
-      </c>
-      <c r="D73">
+      <c r="C73" s="9">
+        <v>2</v>
+      </c>
+      <c r="D73" s="9">
         <v>3</v>
       </c>
-      <c r="E73">
-        <v>2</v>
-      </c>
-      <c r="F73">
+      <c r="E73" s="9">
+        <v>2</v>
+      </c>
+      <c r="F73" s="9">
         <v>1</v>
       </c>
       <c r="G73" s="8"/>
@@ -2104,16 +2104,16 @@
       <c r="B74" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C74">
-        <v>2</v>
-      </c>
-      <c r="D74">
+      <c r="C74" s="9">
+        <v>2</v>
+      </c>
+      <c r="D74" s="9">
         <v>3</v>
       </c>
-      <c r="E74">
-        <v>2</v>
-      </c>
-      <c r="F74">
+      <c r="E74" s="9">
+        <v>2</v>
+      </c>
+      <c r="F74" s="9">
         <v>2</v>
       </c>
       <c r="G74" s="8"/>
@@ -2125,16 +2125,16 @@
       <c r="B75" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C75">
-        <v>2</v>
-      </c>
-      <c r="D75">
-        <v>1</v>
-      </c>
-      <c r="E75">
-        <v>1</v>
-      </c>
-      <c r="F75">
+      <c r="C75" s="9">
+        <v>2</v>
+      </c>
+      <c r="D75" s="9">
+        <v>1</v>
+      </c>
+      <c r="E75" s="9">
+        <v>1</v>
+      </c>
+      <c r="F75" s="9">
         <v>2</v>
       </c>
       <c r="G75" s="8"/>
@@ -2146,16 +2146,16 @@
       <c r="B76" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C76">
-        <v>2</v>
-      </c>
-      <c r="D76">
+      <c r="C76" s="9">
+        <v>2</v>
+      </c>
+      <c r="D76" s="9">
         <v>4</v>
       </c>
-      <c r="E76">
-        <v>2</v>
-      </c>
-      <c r="F76">
+      <c r="E76" s="9">
+        <v>2</v>
+      </c>
+      <c r="F76" s="9">
         <v>1</v>
       </c>
       <c r="G76" s="8"/>
@@ -2167,16 +2167,16 @@
       <c r="B77" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C77">
-        <v>1</v>
-      </c>
-      <c r="D77">
-        <v>2</v>
-      </c>
-      <c r="E77">
-        <v>1</v>
-      </c>
-      <c r="F77">
+      <c r="C77" s="9">
+        <v>1</v>
+      </c>
+      <c r="D77" s="9">
+        <v>2</v>
+      </c>
+      <c r="E77" s="9">
+        <v>1</v>
+      </c>
+      <c r="F77" s="9">
         <v>2</v>
       </c>
       <c r="G77" s="8"/>
@@ -2188,16 +2188,16 @@
       <c r="B78" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C78">
-        <v>1</v>
-      </c>
-      <c r="D78">
+      <c r="C78" s="9">
+        <v>1</v>
+      </c>
+      <c r="D78" s="9">
         <v>4</v>
       </c>
-      <c r="E78">
-        <v>2</v>
-      </c>
-      <c r="F78">
+      <c r="E78" s="9">
+        <v>2</v>
+      </c>
+      <c r="F78" s="9">
         <v>2</v>
       </c>
       <c r="G78" s="8"/>
@@ -2209,16 +2209,16 @@
       <c r="B79" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C79">
-        <v>2</v>
-      </c>
-      <c r="D79">
-        <v>2</v>
-      </c>
-      <c r="E79">
-        <v>1</v>
-      </c>
-      <c r="F79">
+      <c r="C79" s="9">
+        <v>2</v>
+      </c>
+      <c r="D79" s="9">
+        <v>2</v>
+      </c>
+      <c r="E79" s="9">
+        <v>1</v>
+      </c>
+      <c r="F79" s="9">
         <v>1</v>
       </c>
       <c r="G79" s="8"/>
@@ -2230,16 +2230,16 @@
       <c r="B80" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C80">
-        <v>1</v>
-      </c>
-      <c r="D80">
+      <c r="C80" s="9">
+        <v>1</v>
+      </c>
+      <c r="D80" s="9">
         <v>4</v>
       </c>
-      <c r="E80">
-        <v>2</v>
-      </c>
-      <c r="F80">
+      <c r="E80" s="9">
+        <v>2</v>
+      </c>
+      <c r="F80" s="9">
         <v>2</v>
       </c>
       <c r="G80" s="8"/>
@@ -2251,16 +2251,16 @@
       <c r="B81" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C81">
-        <v>1</v>
-      </c>
-      <c r="D81">
+      <c r="C81" s="9">
+        <v>1</v>
+      </c>
+      <c r="D81" s="9">
         <v>3</v>
       </c>
-      <c r="E81">
-        <v>2</v>
-      </c>
-      <c r="F81">
+      <c r="E81" s="9">
+        <v>2</v>
+      </c>
+      <c r="F81" s="9">
         <v>1</v>
       </c>
       <c r="G81" s="8"/>
@@ -2272,16 +2272,16 @@
       <c r="B82" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C82">
-        <v>2</v>
-      </c>
-      <c r="D82">
-        <v>2</v>
-      </c>
-      <c r="E82">
-        <v>1</v>
-      </c>
-      <c r="F82">
+      <c r="C82" s="9">
+        <v>2</v>
+      </c>
+      <c r="D82" s="9">
+        <v>2</v>
+      </c>
+      <c r="E82" s="9">
+        <v>1</v>
+      </c>
+      <c r="F82" s="9">
         <v>2</v>
       </c>
       <c r="G82" s="8"/>

</xml_diff>